<commit_message>
Fix browser export timezone and refresh dashboard UI
</commit_message>
<xml_diff>
--- a/input/shifts.xlsx
+++ b/input/shifts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rawli\OneDrive\Desktop\AttendanceAutomation\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE225BF6-63BE-44FC-9EF7-B02961B31F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D032E20E-48C0-494B-9BB4-10B06C123C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,8 +17,17 @@
     <sheet name="Department_Rules" sheetId="2" r:id="rId2"/>
     <sheet name="Shifts_Config" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -27,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="254">
   <si>
     <t xml:space="preserve">  FO_ROTATING = Front Office rotating (8am-5pm / 9am-6pm / 10am-7pm / 11am-8pm / 6:30pm-8am night). Script picks closest shift per punch.</t>
   </si>
@@ -786,13 +795,16 @@
   </si>
   <si>
     <t>14:00</t>
+  </si>
+  <si>
+    <t>Default_Day,Day_11to8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -815,6 +827,13 @@
     <font>
       <sz val="10"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="9">
@@ -860,7 +879,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -883,11 +902,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBDC3C7"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBDC3C7"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -932,6 +962,10 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3074,7 +3108,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -3361,8 +3395,17 @@
         <v>213</v>
       </c>
     </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A36" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="B36" s="17" t="s">
+        <v>253</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>